<commit_message>
Record the 2026-09-02 live FIFO of 30 and persist the daily cursor.
Batch API Agent - 9/2/26 (694): 18 Success headers 9757-9774, 10 Fail, 2 HOLD bills after vendor-alias retry. Cursor advanced to 2026-08-05T04:26:33Z. Treyce emailed from accountspayable@.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-02.xlsx
+++ b/runs/AP-run-2026-09-02.xlsx
@@ -619,27 +619,33 @@
           <t>NTEX Electric Inc.</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr"/>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>17-2557</t>
+        </is>
+      </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
           <t>2026-08-01</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="n"/>
       <c r="E3" s="2" t="n">
-        <v>1565.34</v>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Fail</t>
+        <v>1694.48</v>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Fail: header create HTTP 400: {"state":"Added","errors":[{"field":"Terms_Code","message":"The Terms Code field is required."},{"field":"Invoice_Due_Date","message":"The Invoice Due Date field is required."},{"field":"Currency","message":"The Currency field is required."},{"field":"Invoice_Number","message":"The Invoice field is required."},{"field":"Vendor","message":"The Vendor field is required."},{"field":"Invoice_Type","message":"The Invoice Type field is required."},{"field":"Transaction_Date","message":"The Transaction Flag status=ai-hold.</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr"/>
+          <t>Header created (Invoice_Type 4). Purchase Order left blank (no-PO or multi-PO or PO not on target). Do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>9765</v>
+      </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26 (694)</t>
@@ -657,7 +663,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>blocked-405</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -667,7 +673,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>ai-hold</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
     </row>
@@ -687,7 +693,7 @@
           <t>2026-07-31</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="n"/>
       <c r="E4" s="2" t="n">
         <v>5403.45</v>
       </c>
@@ -751,7 +757,7 @@
           <t>2026-07-31</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="n"/>
       <c r="E5" s="2" t="n"/>
       <c r="F5" s="3" t="inlineStr">
         <is>
@@ -800,7 +806,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Emily Keith</t>
+          <t>Morgan Steel</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -826,10 +832,14 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Fail: vendor missing on live for Emily Keith (looked up by vendor name). Will not invent a vendor/remit-to ID. Flag status=ai-hold.</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr"/>
+          <t>Fail/already exists (id 9752) Morgan Steel 128249 on live. Will not recreate.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>9752</t>
+        </is>
+      </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26 (694)</t>
@@ -864,7 +874,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Emily Keith</t>
+          <t>Morgan Steel</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -879,21 +889,25 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>5420</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>Fail</t>
+          <t>58718</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>13404.84</v>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Fail: vendor missing on live for Emily Keith (looked up by vendor name). Will not invent a vendor/remit-to ID. Flag status=ai-hold.</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr"/>
+          <t>Header created (Invoice_Type 3). Header PO set. Select Receipts via API not implemented without an Editable receipt action; do not type Add Item. Select Receipts: 1 receipt(s) matched by part/PO-WO/slip (not first qty). Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>9766</v>
+      </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26 (694)</t>
@@ -911,7 +925,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>blocked-405</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -921,7 +935,7 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>ai-hold</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
     </row>
@@ -941,7 +955,7 @@
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr"/>
+      <c r="D8" s="2" t="n"/>
       <c r="E8" s="2" t="n">
         <v>2386.55</v>
       </c>
@@ -992,7 +1006,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Accounts Receivable</t>
+          <t>American Bearing Company</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1005,7 +1019,7 @@
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr"/>
+      <c r="D9" s="2" t="n"/>
       <c r="E9" s="2" t="n">
         <v>4993.22</v>
       </c>
@@ -1016,10 +1030,14 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Fail: vendor missing on live for Accounts Receivable (looked up by vendor name). Will not invent a vendor/remit-to ID. Flag status=ai-hold.</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr"/>
+          <t>Fail/already exists (id 9755) American Bearing 296567 / PO 58595. Will not recreate.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>9755</t>
+        </is>
+      </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26 (694)</t>
@@ -1054,7 +1072,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Greg Tunnell - Crosslink Powder Coating</t>
+          <t>Crosslink Powder Coating</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1067,7 +1085,7 @@
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="n"/>
       <c r="E10" s="2" t="n">
         <v>1252.18</v>
       </c>
@@ -1078,11 +1096,13 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Fail/already exists (id 9756) Flag status=ai-hold.</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="n">
-        <v>9756</v>
+          <t>Fail/already exists (id 9756) Crosslink 27756 / PO 58723. Will not recreate.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>9756</t>
+        </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -1131,7 +1151,7 @@
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr"/>
+      <c r="D11" s="2" t="n"/>
       <c r="E11" s="2" t="n">
         <v>1107.57</v>
       </c>
@@ -1195,7 +1215,7 @@
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="n"/>
       <c r="E12" s="2" t="n">
         <v>8697.370000000001</v>
       </c>
@@ -1209,7 +1229,7 @@
           <t>Fail: vendor missing on live for ENGIE Resources LLC (looked up by vendor name). Will not invent a vendor/remit-to ID. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="n"/>
       <c r="I12" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26 (694)</t>
@@ -1244,12 +1264,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>billingdal@grmdocument.com</t>
+          <t>GRM Information Management Services</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>13010065</t>
+          <t>00012913</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1257,21 +1277,23 @@
           <t>2026-07-31</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr"/>
+      <c r="D13" s="2" t="n"/>
       <c r="E13" s="2" t="n">
-        <v>47.69</v>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>Fail</t>
+        <v>189.78</v>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Fail: vendor missing on live for billingdal@grmdocument.com (looked up by vendor name). Will not invent a vendor/remit-to ID. Flag status=ai-hold.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr"/>
+          <t>Header created (Invoice_Type 4). Purchase Order left blank (no-PO or multi-PO or PO not on target). Do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>9767</v>
+      </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26 (694)</t>
@@ -1279,7 +1301,7 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Account Maintenance Fee 22.6800 1.00 22.68; Check Processing Fee on check #18302 25.0000 1.00 25.00</t>
+          <t>Account Maintenance Fee 22.68; Check Processing Fee 25.00</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1289,7 +1311,7 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>blocked-405</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
@@ -1299,7 +1321,7 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>ai-hold</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
     </row>
@@ -1319,7 +1341,7 @@
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="n"/>
       <c r="E14" s="2" t="n">
         <v>1265.3</v>
       </c>
@@ -1370,7 +1392,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>autotask@kloecknermetals.com</t>
+          <t>Kloeckner Metals Corporation</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1378,26 +1400,32 @@
           <t>15206040</t>
         </is>
       </c>
-      <c r="C15" s="2" t="n"/>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>25576511</t>
+          <t>58728</t>
         </is>
       </c>
       <c r="E15" s="2" t="n">
         <v>7167</v>
       </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>Fail</t>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Fail: vendor missing on live for autotask@kloecknermetals.com (looked up by vendor name). Will not invent a vendor/remit-to ID. Flag status=ai-hold.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr"/>
+          <t>Header created (Invoice_Type 3). Header PO set. Select Receipts via API not implemented without an Editable receipt action; do not type Add Item. Select Receipts: 1 receipt(s) matched by part/PO-WO/slip (not first qty). Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>9768</v>
+      </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26 (694)</t>
@@ -1415,7 +1443,7 @@
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>blocked-405</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
@@ -1425,7 +1453,7 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>ai-hold</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1596,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Ryerson Invoice - Do Not Reply</t>
+          <t>Joseph T. Ryerson &amp; Son, Inc</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1589,17 +1617,19 @@
       <c r="E18" s="2" t="n">
         <v>480.26</v>
       </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>HOLD: no receipts after slip # / part / qty / PO line search (invoice 9306966730). Will not guess a qty-only slip. Flag status=ai-hold.</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr"/>
+          <t>Header created (Invoice_Type 3). Header PO set. Select Receipts via API not implemented without an Editable receipt action; do not type Add Item. Select Receipts: 1 receipt(s) matched by part/PO-WO/slip (not first qty). Post Additional Charge Purchase Price Variance 4.91 (signed; negative allowed). Additional Charge Purchase Price Variance 4.91 (signed; |var| 4.91 is 1.0% of invoice total and bill PPV 4.91 is under $100) Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>9771</v>
+      </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26 (694)</t>
@@ -1607,17 +1637,17 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Shipping Type Truck; Fuel Surcharge 0.33 USD 0.33; Remittances are received by a bank acting as a clearing agency without authority; notation regarding payment in full or settlement, the bank shall deposit such re; shall be effective to alter or add to Ryerson's standard conditions and terms of</t>
+          <t>Fuel Surcharge 0.33</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>5.24</t>
+          <t>4.91</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>blocked-405</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
@@ -1627,7 +1657,7 @@
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>ai-hold</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
     </row>
@@ -1665,7 +1695,7 @@
           <t>HOLD: no receipts after slip # / part / qty / PO line search (invoice 69440053). Will not guess a qty-only slip. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="n"/>
       <c r="I19" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26 (694)</t>
@@ -1700,7 +1730,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Beth.Watkins@kloeckner.com</t>
+          <t>Kloeckner Metals Corporation</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1724,10 +1754,14 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Fail: vendor missing on live for Beth.Watkins@kloeckner.com (looked up by vendor name). Will not invent a vendor/remit-to ID. Flag status=ai-hold.</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr"/>
+          <t>Fail/already exists (id 9170) Kloeckner 15205174. Will not recreate.</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>9170</t>
+        </is>
+      </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26 (694)</t>
@@ -1762,7 +1796,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Nanci Meza</t>
+          <t>Kloeckner Metals Corporation</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1786,10 +1820,14 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Fail: vendor missing on live for Nanci Meza (looked up by vendor name). Will not invent a vendor/remit-to ID. Flag status=ai-hold.</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr"/>
+          <t>Fail/already exists (id 9170) Kloeckner 15205174 (duplicate email). Will not recreate.</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>9170</t>
+        </is>
+      </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26 (694)</t>
@@ -1824,30 +1862,40 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>DoNotReply@altparts.com</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr"/>
+          <t>Alternative Parts Inc</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>0097416-IN</t>
+        </is>
+      </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>58832</t>
+        </is>
+      </c>
       <c r="E22" s="2" t="n">
         <v>1765.44</v>
       </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>Fail</t>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Fail: vendor missing on live for DoNotReply@altparts.com (looked up by vendor name). Will not invent a vendor/remit-to ID. Flag status=ai-hold.</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr"/>
+          <t>Header created (Invoice_Type 3). Header PO set from live PO 58832. Select Receipts via API not implemented; do not type Add Item. Fees go to Additional Charge Fees and surcharges (Freight 36.44). Attach status=blocked-405. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>9774</v>
+      </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26 (694)</t>
@@ -1855,7 +1903,7 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Freight Account; Freight 36.44; In addition to the above ‘API Returned Products,’ optics must be in the original</t>
+          <t>Freight 36.44</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -1865,7 +1913,7 @@
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>blocked-405</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
@@ -1875,7 +1923,7 @@
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>ai-hold</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
     </row>
@@ -1895,7 +1943,7 @@
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr"/>
+      <c r="D23" s="2" t="n"/>
       <c r="E23" s="2" t="n">
         <v>422.87</v>
       </c>
@@ -1906,11 +1954,13 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Header created (Invoice_Type 4). Purchase Order left blank (no-PO or multi-PO or PO not on target). Do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405. Flag status=entered-in-ai.</t>
-        </is>
-      </c>
-      <c r="H23" s="2" t="n">
-        <v>9761</v>
+          <t>Success already posted as 9761 using customer # 02627782; printed invoice is 66623661. Will not recreate.</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>9761</t>
+        </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
@@ -1946,30 +1996,40 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>accounting2@sss-steel.com</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr"/>
+          <t>Tube Supply</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>01175961</t>
+        </is>
+      </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>58809</t>
+        </is>
+      </c>
       <c r="E24" s="2" t="n">
         <v>2140.74</v>
       </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>Fail</t>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Fail: vendor missing on live for accounting2@sss-steel.com (looked up by vendor name). Will not invent a vendor/remit-to ID. Flag status=ai-hold.</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr"/>
+          <t>Header created (Invoice_Type 3). Header PO set. Select Receipts via API not implemented without an Editable receipt action; do not type Add Item. Select Receipts: 1 receipt(s) matched by part/PO-WO/slip (not first qty). Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>9769</v>
+      </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26 (694)</t>
@@ -1977,7 +2037,7 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>SHIPPING POINT</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -1987,7 +2047,7 @@
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>blocked-405</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
@@ -1997,19 +2057,19 @@
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>ai-hold</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Sandi Ehlers</t>
+          <t>Lavanture Products</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>1786258</t>
+          <t>SV1426672</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -2017,21 +2077,27 @@
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr"/>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>58843</t>
+        </is>
+      </c>
       <c r="E25" s="2" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>Fail</t>
+        <v>38.04</v>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Fail: vendor missing on live for Sandi Ehlers (looked up by vendor name). Will not invent a vendor/remit-to ID. Flag status=ai-hold.</t>
-        </is>
-      </c>
-      <c r="H25" s="2" t="inlineStr"/>
+          <t>Header created (Invoice_Type 3). Header PO set. Select Receipts via API not implemented without an Editable receipt action; do not type Add Item. Select Receipts: 1 receipt(s) matched by part/PO-WO/slip (not first qty). Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>9770</v>
+      </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26 (694)</t>
@@ -2039,7 +2105,7 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>Freight</t>
+          <t>Freight 15.08</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -2049,7 +2115,7 @@
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>blocked-405</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
@@ -2059,14 +2125,14 @@
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>ai-hold</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Bookkeeper</t>
+          <t>McQueary Industries</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2094,11 +2160,13 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Header created (Invoice_Type 3). Header PO set. Select Receipts via API not implemented without an Editable receipt action; do not type Add Item. Select Receipts: 1 receipt(s) matched by part/PO-WO/slip (not first qty). Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405. Flag status=entered-in-ai.</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="n">
-        <v>9762</v>
+          <t>Success already posted as 9762 using filename 14152; printed invoice is 08-30336. Will not recreate.</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>9762</t>
+        </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
@@ -2155,17 +2223,19 @@
       <c r="E27" s="2" t="n">
         <v>1043.93</v>
       </c>
-      <c r="F27" s="5" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>HOLD: no receipts after slip # / part / qty / PO line search (invoice 816653). Will not guess a qty-only slip. Flag status=ai-hold.</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="inlineStr"/>
+          <t>Header created (Invoice_Type 3). Header PO set. Select Receipts via API not implemented without an Editable receipt action; do not type Add Item. Select Receipts: 1 receipt(s) matched by part/PO-WO/slip (not first qty). Post Additional Charge Purchase Price Variance 0.02 (signed; negative allowed). Additional Charge Purchase Price Variance 0.02 (signed; |var| 0.02 is 0.0% of invoice total and bill PPV 0.02 is under $100) Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>9772</v>
+      </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26 (694)</t>
@@ -2173,17 +2243,17 @@
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>Sub-Total Discounts Tax Handling Freight Misc TOTAL-DUE; Misc 91 SHIPPING &amp; HANDLING SURCHARGE 60.00</t>
+          <t>Shipping &amp; Handling Surcharge 60.00</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>60.02</t>
+          <t>0.02</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>blocked-405</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
@@ -2193,7 +2263,7 @@
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>ai-hold</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
     </row>
@@ -2221,17 +2291,19 @@
       <c r="E28" s="2" t="n">
         <v>613.62</v>
       </c>
-      <c r="F28" s="5" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>HOLD: no receipts after slip # / part / qty / PO line search (invoice 816654). Will not guess a qty-only slip. Flag status=ai-hold.</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr"/>
+          <t>Header created (Invoice_Type 3). Header PO set. Select Receipts via API not implemented without an Editable receipt action; do not type Add Item. Select Receipts: 1 receipt(s) matched by part/PO-WO/slip (not first qty). Post Additional Charge Purchase Price Variance 0.18 (signed; negative allowed). Additional Charge Purchase Price Variance 0.18 (signed; |var| 0.18 is 0.0% of invoice total and bill PPV 0.18 is under $100) Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>9773</v>
+      </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26 (694)</t>
@@ -2239,7 +2311,7 @@
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>Sub-Total Discounts Tax Handling Freight Misc TOTAL-DUE</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
@@ -2249,7 +2321,7 @@
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>blocked-405</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
@@ -2259,7 +2331,7 @@
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>ai-hold</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
     </row>
@@ -2279,7 +2351,7 @@
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr"/>
+      <c r="D29" s="2" t="n"/>
       <c r="E29" s="2" t="n">
         <v>2030.8</v>
       </c>
@@ -2361,7 +2433,7 @@
           <t>HOLD: price does not match (23.3% of invoice total). Do not post PPV. Purchasing must unreceive, change the PO price, and re-receive. Comment the PO line for @Shawn McKibben. Do not alter receipt unit price in GI. @Shawn McKibben price does not match. Purchasing must unreceive, change the PO price, and re-receive. Do not alter receipt unit price in GI (breaks WO cost, material cost, and PO clearing). Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr"/>
+      <c r="H30" s="2" t="n"/>
       <c r="I30" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26 (694)</t>
@@ -2467,14 +2539,14 @@
           <t>UniFirstStatements@UniFirst.com</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr"/>
+      <c r="B32" s="2" t="n"/>
       <c r="C32" s="2" t="inlineStr">
         <is>
           <t>2026-08-02</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr"/>
-      <c r="E32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="n"/>
+      <c r="E32" s="2" t="n"/>
       <c r="F32" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -2485,7 +2557,7 @@
           <t>HOLD: statement. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="n"/>
       <c r="I32" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -2523,14 +2595,14 @@
           <t>amazon.com</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr"/>
+      <c r="B33" s="2" t="n"/>
       <c r="C33" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr"/>
-      <c r="E33" s="2" t="inlineStr"/>
+      <c r="D33" s="2" t="n"/>
+      <c r="E33" s="2" t="n"/>
       <c r="F33" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -2541,7 +2613,7 @@
           <t>HOLD: not-a-bill. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr"/>
+      <c r="H33" s="2" t="n"/>
       <c r="I33" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -2589,8 +2661,8 @@
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr"/>
-      <c r="E34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="n"/>
+      <c r="E34" s="2" t="n"/>
       <c r="F34" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -2601,7 +2673,7 @@
           <t>HOLD: CHECK STOP. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr"/>
+      <c r="H34" s="2" t="n"/>
       <c r="I34" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -2639,14 +2711,14 @@
           <t>Shaw, Linda</t>
         </is>
       </c>
-      <c r="B35" s="2" t="inlineStr"/>
+      <c r="B35" s="2" t="n"/>
       <c r="C35" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr"/>
-      <c r="E35" s="2" t="inlineStr"/>
+      <c r="D35" s="2" t="n"/>
+      <c r="E35" s="2" t="n"/>
       <c r="F35" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -2657,7 +2729,7 @@
           <t>HOLD: not-a-bill. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H35" s="2" t="inlineStr"/>
+      <c r="H35" s="2" t="n"/>
       <c r="I35" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -2695,14 +2767,14 @@
           <t>Spectrum Business</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr"/>
+      <c r="B36" s="2" t="n"/>
       <c r="C36" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr"/>
-      <c r="E36" s="2" t="inlineStr"/>
+      <c r="D36" s="2" t="n"/>
+      <c r="E36" s="2" t="n"/>
       <c r="F36" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -2713,7 +2785,7 @@
           <t>HOLD: not-a-bill. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr"/>
+      <c r="H36" s="2" t="n"/>
       <c r="I36" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -2751,14 +2823,14 @@
           <t>CertSOLV on behalf of Engie Resources LLC</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr"/>
+      <c r="B37" s="2" t="n"/>
       <c r="C37" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr"/>
-      <c r="E37" s="2" t="inlineStr"/>
+      <c r="D37" s="2" t="n"/>
+      <c r="E37" s="2" t="n"/>
       <c r="F37" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -2769,7 +2841,7 @@
           <t>HOLD: not-a-bill. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H37" s="2" t="inlineStr"/>
+      <c r="H37" s="2" t="n"/>
       <c r="I37" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -2807,14 +2879,14 @@
           <t>Nanci Meza</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr"/>
+      <c r="B38" s="2" t="n"/>
       <c r="C38" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr"/>
-      <c r="E38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="n"/>
+      <c r="E38" s="2" t="n"/>
       <c r="F38" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -2825,7 +2897,7 @@
           <t>HOLD: not-a-bill. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr"/>
+      <c r="H38" s="2" t="n"/>
       <c r="I38" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -2863,14 +2935,14 @@
           <t>Amazon Business</t>
         </is>
       </c>
-      <c r="B39" s="2" t="inlineStr"/>
+      <c r="B39" s="2" t="n"/>
       <c r="C39" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr"/>
-      <c r="E39" s="2" t="inlineStr"/>
+      <c r="D39" s="2" t="n"/>
+      <c r="E39" s="2" t="n"/>
       <c r="F39" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -2881,7 +2953,7 @@
           <t>HOLD: not-a-bill. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H39" s="2" t="inlineStr"/>
+      <c r="H39" s="2" t="n"/>
       <c r="I39" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -2919,14 +2991,14 @@
           <t>Pocketbook</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr"/>
+      <c r="B40" s="2" t="n"/>
       <c r="C40" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr"/>
-      <c r="E40" s="2" t="inlineStr"/>
+      <c r="D40" s="2" t="n"/>
+      <c r="E40" s="2" t="n"/>
       <c r="F40" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -2937,7 +3009,7 @@
           <t>HOLD: not-a-bill. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr"/>
+      <c r="H40" s="2" t="n"/>
       <c r="I40" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -2975,14 +3047,14 @@
           <t>Yasaman Morshed</t>
         </is>
       </c>
-      <c r="B41" s="2" t="inlineStr"/>
+      <c r="B41" s="2" t="n"/>
       <c r="C41" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D41" s="2" t="inlineStr"/>
-      <c r="E41" s="2" t="inlineStr"/>
+      <c r="D41" s="2" t="n"/>
+      <c r="E41" s="2" t="n"/>
       <c r="F41" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -2993,7 +3065,7 @@
           <t>HOLD: not-a-bill. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H41" s="2" t="inlineStr"/>
+      <c r="H41" s="2" t="n"/>
       <c r="I41" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -3031,14 +3103,14 @@
           <t>AMERICAN QUALITY POWDER COATING</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr"/>
+      <c r="B42" s="2" t="n"/>
       <c r="C42" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr"/>
-      <c r="E42" s="2" t="inlineStr"/>
+      <c r="D42" s="2" t="n"/>
+      <c r="E42" s="2" t="n"/>
       <c r="F42" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -3049,7 +3121,7 @@
           <t>HOLD: not-a-bill. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr"/>
+      <c r="H42" s="2" t="n"/>
       <c r="I42" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -3087,14 +3159,14 @@
           <t>AMERICAN QUALITY POWDER COATING</t>
         </is>
       </c>
-      <c r="B43" s="2" t="inlineStr"/>
+      <c r="B43" s="2" t="n"/>
       <c r="C43" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr"/>
-      <c r="E43" s="2" t="inlineStr"/>
+      <c r="D43" s="2" t="n"/>
+      <c r="E43" s="2" t="n"/>
       <c r="F43" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -3105,7 +3177,7 @@
           <t>HOLD: not-a-bill. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H43" s="2" t="inlineStr"/>
+      <c r="H43" s="2" t="n"/>
       <c r="I43" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -3143,14 +3215,14 @@
           <t>AMERICAN QUALITY POWDER COATING</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr"/>
+      <c r="B44" s="2" t="n"/>
       <c r="C44" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D44" s="2" t="inlineStr"/>
-      <c r="E44" s="2" t="inlineStr"/>
+      <c r="D44" s="2" t="n"/>
+      <c r="E44" s="2" t="n"/>
       <c r="F44" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -3161,7 +3233,7 @@
           <t>HOLD: not-a-bill. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H44" s="2" t="inlineStr"/>
+      <c r="H44" s="2" t="n"/>
       <c r="I44" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -3199,14 +3271,14 @@
           <t>AMERICAN QUALITY POWDER COATING</t>
         </is>
       </c>
-      <c r="B45" s="2" t="inlineStr"/>
+      <c r="B45" s="2" t="n"/>
       <c r="C45" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr"/>
-      <c r="E45" s="2" t="inlineStr"/>
+      <c r="D45" s="2" t="n"/>
+      <c r="E45" s="2" t="n"/>
       <c r="F45" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -3217,7 +3289,7 @@
           <t>HOLD: not-a-bill. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H45" s="2" t="inlineStr"/>
+      <c r="H45" s="2" t="n"/>
       <c r="I45" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -3255,14 +3327,14 @@
           <t>Accounts Payable</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr"/>
+      <c r="B46" s="2" t="n"/>
       <c r="C46" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D46" s="2" t="inlineStr"/>
-      <c r="E46" s="2" t="inlineStr"/>
+      <c r="D46" s="2" t="n"/>
+      <c r="E46" s="2" t="n"/>
       <c r="F46" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -3273,7 +3345,7 @@
           <t>HOLD: not-a-bill. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr"/>
+      <c r="H46" s="2" t="n"/>
       <c r="I46" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -3311,14 +3383,14 @@
           <t>Accounts Receivables</t>
         </is>
       </c>
-      <c r="B47" s="2" t="inlineStr"/>
+      <c r="B47" s="2" t="n"/>
       <c r="C47" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D47" s="2" t="inlineStr"/>
-      <c r="E47" s="2" t="inlineStr"/>
+      <c r="D47" s="2" t="n"/>
+      <c r="E47" s="2" t="n"/>
       <c r="F47" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -3329,7 +3401,7 @@
           <t>HOLD: statement. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H47" s="2" t="inlineStr"/>
+      <c r="H47" s="2" t="n"/>
       <c r="I47" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -3367,14 +3439,14 @@
           <t>Giovanny</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr"/>
+      <c r="B48" s="2" t="n"/>
       <c r="C48" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D48" s="2" t="inlineStr"/>
-      <c r="E48" s="2" t="inlineStr"/>
+      <c r="D48" s="2" t="n"/>
+      <c r="E48" s="2" t="n"/>
       <c r="F48" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -3385,7 +3457,7 @@
           <t>HOLD: pod. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H48" s="2" t="inlineStr"/>
+      <c r="H48" s="2" t="n"/>
       <c r="I48" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -3423,14 +3495,14 @@
           <t>Giovanny</t>
         </is>
       </c>
-      <c r="B49" s="2" t="inlineStr"/>
+      <c r="B49" s="2" t="n"/>
       <c r="C49" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D49" s="2" t="inlineStr"/>
-      <c r="E49" s="2" t="inlineStr"/>
+      <c r="D49" s="2" t="n"/>
+      <c r="E49" s="2" t="n"/>
       <c r="F49" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -3441,7 +3513,7 @@
           <t>HOLD: pod. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H49" s="2" t="inlineStr"/>
+      <c r="H49" s="2" t="n"/>
       <c r="I49" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -3479,14 +3551,14 @@
           <t>Giovanny</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr"/>
+      <c r="B50" s="2" t="n"/>
       <c r="C50" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D50" s="2" t="inlineStr"/>
-      <c r="E50" s="2" t="inlineStr"/>
+      <c r="D50" s="2" t="n"/>
+      <c r="E50" s="2" t="n"/>
       <c r="F50" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -3497,7 +3569,7 @@
           <t>HOLD: pod. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H50" s="2" t="inlineStr"/>
+      <c r="H50" s="2" t="n"/>
       <c r="I50" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -3535,14 +3607,14 @@
           <t>Nanci Meza</t>
         </is>
       </c>
-      <c r="B51" s="2" t="inlineStr"/>
+      <c r="B51" s="2" t="n"/>
       <c r="C51" s="2" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="D51" s="2" t="inlineStr"/>
-      <c r="E51" s="2" t="inlineStr"/>
+      <c r="D51" s="2" t="n"/>
+      <c r="E51" s="2" t="n"/>
       <c r="F51" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -3553,7 +3625,7 @@
           <t>HOLD: not-a-bill. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H51" s="2" t="inlineStr"/>
+      <c r="H51" s="2" t="n"/>
       <c r="I51" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -3591,14 +3663,14 @@
           <t>OLP5190@WASTECONNECTIONS.COM</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr"/>
+      <c r="B52" s="2" t="n"/>
       <c r="C52" s="2" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="D52" s="2" t="inlineStr"/>
-      <c r="E52" s="2" t="inlineStr"/>
+      <c r="D52" s="2" t="n"/>
+      <c r="E52" s="2" t="n"/>
       <c r="F52" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -3609,7 +3681,7 @@
           <t>HOLD: not-a-bill. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H52" s="2" t="inlineStr"/>
+      <c r="H52" s="2" t="n"/>
       <c r="I52" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -3647,14 +3719,14 @@
           <t>Andrea Sylvester</t>
         </is>
       </c>
-      <c r="B53" s="2" t="inlineStr"/>
+      <c r="B53" s="2" t="n"/>
       <c r="C53" s="2" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="D53" s="2" t="inlineStr"/>
-      <c r="E53" s="2" t="inlineStr"/>
+      <c r="D53" s="2" t="n"/>
+      <c r="E53" s="2" t="n"/>
       <c r="F53" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -3665,7 +3737,7 @@
           <t>HOLD: statement. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H53" s="2" t="inlineStr"/>
+      <c r="H53" s="2" t="n"/>
       <c r="I53" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -3703,14 +3775,14 @@
           <t>Michelle Dalton</t>
         </is>
       </c>
-      <c r="B54" s="2" t="inlineStr"/>
+      <c r="B54" s="2" t="n"/>
       <c r="C54" s="2" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="D54" s="2" t="inlineStr"/>
-      <c r="E54" s="2" t="inlineStr"/>
+      <c r="D54" s="2" t="n"/>
+      <c r="E54" s="2" t="n"/>
       <c r="F54" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -3721,7 +3793,7 @@
           <t>HOLD: not-a-bill. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H54" s="2" t="inlineStr"/>
+      <c r="H54" s="2" t="n"/>
       <c r="I54" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -3759,14 +3831,14 @@
           <t>Nanci Meza</t>
         </is>
       </c>
-      <c r="B55" s="2" t="inlineStr"/>
+      <c r="B55" s="2" t="n"/>
       <c r="C55" s="2" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr"/>
-      <c r="E55" s="2" t="inlineStr"/>
+      <c r="D55" s="2" t="n"/>
+      <c r="E55" s="2" t="n"/>
       <c r="F55" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -3777,7 +3849,7 @@
           <t>HOLD: not-a-bill. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H55" s="2" t="inlineStr"/>
+      <c r="H55" s="2" t="n"/>
       <c r="I55" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -3815,14 +3887,14 @@
           <t>Nanci Meza</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr"/>
+      <c r="B56" s="2" t="n"/>
       <c r="C56" s="2" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="D56" s="2" t="inlineStr"/>
-      <c r="E56" s="2" t="inlineStr"/>
+      <c r="D56" s="2" t="n"/>
+      <c r="E56" s="2" t="n"/>
       <c r="F56" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -3833,7 +3905,7 @@
           <t>HOLD: not-a-bill. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H56" s="2" t="inlineStr"/>
+      <c r="H56" s="2" t="n"/>
       <c r="I56" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -3871,14 +3943,14 @@
           <t>Giovanny</t>
         </is>
       </c>
-      <c r="B57" s="2" t="inlineStr"/>
+      <c r="B57" s="2" t="n"/>
       <c r="C57" s="2" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="D57" s="2" t="inlineStr"/>
-      <c r="E57" s="2" t="inlineStr"/>
+      <c r="D57" s="2" t="n"/>
+      <c r="E57" s="2" t="n"/>
       <c r="F57" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -3889,7 +3961,7 @@
           <t>HOLD: pod. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H57" s="2" t="inlineStr"/>
+      <c r="H57" s="2" t="n"/>
       <c r="I57" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -3927,14 +3999,14 @@
           <t>Giovanny</t>
         </is>
       </c>
-      <c r="B58" s="2" t="inlineStr"/>
+      <c r="B58" s="2" t="n"/>
       <c r="C58" s="2" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="D58" s="2" t="inlineStr"/>
-      <c r="E58" s="2" t="inlineStr"/>
+      <c r="D58" s="2" t="n"/>
+      <c r="E58" s="2" t="n"/>
       <c r="F58" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -3945,7 +4017,7 @@
           <t>HOLD: pod. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H58" s="2" t="inlineStr"/>
+      <c r="H58" s="2" t="n"/>
       <c r="I58" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -3983,14 +4055,14 @@
           <t>Credit Department</t>
         </is>
       </c>
-      <c r="B59" s="2" t="inlineStr"/>
+      <c r="B59" s="2" t="n"/>
       <c r="C59" s="2" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="D59" s="2" t="inlineStr"/>
-      <c r="E59" s="2" t="inlineStr"/>
+      <c r="D59" s="2" t="n"/>
+      <c r="E59" s="2" t="n"/>
       <c r="F59" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -4001,7 +4073,7 @@
           <t>HOLD: not-a-bill. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H59" s="2" t="inlineStr"/>
+      <c r="H59" s="2" t="n"/>
       <c r="I59" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -4039,14 +4111,14 @@
           <t>Accounts Payable</t>
         </is>
       </c>
-      <c r="B60" s="2" t="inlineStr"/>
+      <c r="B60" s="2" t="n"/>
       <c r="C60" s="2" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="D60" s="2" t="inlineStr"/>
-      <c r="E60" s="2" t="inlineStr"/>
+      <c r="D60" s="2" t="n"/>
+      <c r="E60" s="2" t="n"/>
       <c r="F60" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -4057,7 +4129,7 @@
           <t>HOLD: not-a-bill. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H60" s="2" t="inlineStr"/>
+      <c r="H60" s="2" t="n"/>
       <c r="I60" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -4095,14 +4167,14 @@
           <t>Spectrum Business</t>
         </is>
       </c>
-      <c r="B61" s="2" t="inlineStr"/>
+      <c r="B61" s="2" t="n"/>
       <c r="C61" s="2" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="D61" s="2" t="inlineStr"/>
-      <c r="E61" s="2" t="inlineStr"/>
+      <c r="D61" s="2" t="n"/>
+      <c r="E61" s="2" t="n"/>
       <c r="F61" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -4113,7 +4185,7 @@
           <t>HOLD: not-a-bill. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H61" s="2" t="inlineStr"/>
+      <c r="H61" s="2" t="n"/>
       <c r="I61" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -4151,14 +4223,14 @@
           <t>Kristen Powers</t>
         </is>
       </c>
-      <c r="B62" s="2" t="inlineStr"/>
+      <c r="B62" s="2" t="n"/>
       <c r="C62" s="2" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="D62" s="2" t="inlineStr"/>
-      <c r="E62" s="2" t="inlineStr"/>
+      <c r="D62" s="2" t="n"/>
+      <c r="E62" s="2" t="n"/>
       <c r="F62" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -4169,7 +4241,7 @@
           <t>HOLD: not-a-bill. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H62" s="2" t="inlineStr"/>
+      <c r="H62" s="2" t="n"/>
       <c r="I62" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -4207,14 +4279,14 @@
           <t>Thermo Fluids</t>
         </is>
       </c>
-      <c r="B63" s="2" t="inlineStr"/>
+      <c r="B63" s="2" t="n"/>
       <c r="C63" s="2" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="D63" s="2" t="inlineStr"/>
-      <c r="E63" s="2" t="inlineStr"/>
+      <c r="D63" s="2" t="n"/>
+      <c r="E63" s="2" t="n"/>
       <c r="F63" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -4225,7 +4297,7 @@
           <t>HOLD: not-a-bill. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H63" s="2" t="inlineStr"/>
+      <c r="H63" s="2" t="n"/>
       <c r="I63" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -4263,14 +4335,14 @@
           <t>Green Valley Compressor LLC</t>
         </is>
       </c>
-      <c r="B64" s="2" t="inlineStr"/>
+      <c r="B64" s="2" t="n"/>
       <c r="C64" s="2" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="D64" s="2" t="inlineStr"/>
-      <c r="E64" s="2" t="inlineStr"/>
+      <c r="D64" s="2" t="n"/>
+      <c r="E64" s="2" t="n"/>
       <c r="F64" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -4281,7 +4353,7 @@
           <t>HOLD: statement. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H64" s="2" t="inlineStr"/>
+      <c r="H64" s="2" t="n"/>
       <c r="I64" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -4319,14 +4391,14 @@
           <t>mwatkins@onealsteel.com</t>
         </is>
       </c>
-      <c r="B65" s="2" t="inlineStr"/>
+      <c r="B65" s="2" t="n"/>
       <c r="C65" s="2" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="D65" s="2" t="inlineStr"/>
-      <c r="E65" s="2" t="inlineStr"/>
+      <c r="D65" s="2" t="n"/>
+      <c r="E65" s="2" t="n"/>
       <c r="F65" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -4337,7 +4409,7 @@
           <t>HOLD: statement. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H65" s="2" t="inlineStr"/>
+      <c r="H65" s="2" t="n"/>
       <c r="I65" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -4375,14 +4447,14 @@
           <t>Riley Armstrong</t>
         </is>
       </c>
-      <c r="B66" s="2" t="inlineStr"/>
+      <c r="B66" s="2" t="n"/>
       <c r="C66" s="2" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="D66" s="2" t="inlineStr"/>
-      <c r="E66" s="2" t="inlineStr"/>
+      <c r="D66" s="2" t="n"/>
+      <c r="E66" s="2" t="n"/>
       <c r="F66" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -4393,7 +4465,7 @@
           <t>HOLD: not-a-bill. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H66" s="2" t="inlineStr"/>
+      <c r="H66" s="2" t="n"/>
       <c r="I66" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>
@@ -4431,14 +4503,14 @@
           <t>ar@onealsteel.com</t>
         </is>
       </c>
-      <c r="B67" s="2" t="inlineStr"/>
+      <c r="B67" s="2" t="n"/>
       <c r="C67" s="2" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="D67" s="2" t="inlineStr"/>
-      <c r="E67" s="2" t="inlineStr"/>
+      <c r="D67" s="2" t="n"/>
+      <c r="E67" s="2" t="n"/>
       <c r="F67" s="5" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -4449,7 +4521,7 @@
           <t>HOLD: payment. Do not create a header. Flag status=ai-hold.</t>
         </is>
       </c>
-      <c r="H67" s="2" t="inlineStr"/>
+      <c r="H67" s="2" t="n"/>
       <c r="I67" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/2/26</t>

</xml_diff>